<commit_message>
Updated partslist rig_v1 + added partslists rig_v2, rig_v2.1
</commit_message>
<xml_diff>
--- a/cad/rig_v1/Partlist.xlsx
+++ b/cad/rig_v1/Partlist.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="83" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="90" uniqueCount="45">
   <si>
     <t>Objekt</t>
   </si>
@@ -42,54 +42,60 @@
     <t>REV.</t>
   </si>
   <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
     <t>4</t>
   </si>
   <si>
-    <t>5</t>
-  </si>
-  <si>
     <t>6</t>
   </si>
   <si>
     <t>3</t>
   </si>
   <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
     <t>2</t>
   </si>
   <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
     <t>12</t>
   </si>
   <si>
+    <t>Winkelsatz_20x20_einfach</t>
+  </si>
+  <si>
+    <t>item_0043784_Klemmwinkel 5_1</t>
+  </si>
+  <si>
+    <t>DIN 603 - M5 x 50</t>
+  </si>
+  <si>
     <t>DIN 9021 - 5,3</t>
   </si>
   <si>
     <t>DIN 1587 - M5</t>
   </si>
   <si>
-    <t>DIN 603 - M5 x 50</t>
-  </si>
-  <si>
-    <t>Winkelsatz_20x20_einfach</t>
-  </si>
-  <si>
     <t>Profil_5_20x20_1500</t>
   </si>
   <si>
@@ -105,34 +111,37 @@
     <t>Zentrierplattensatz_5</t>
   </si>
   <si>
+    <t>Dummy</t>
+  </si>
+  <si>
+    <t>Boden</t>
+  </si>
+  <si>
     <t>Profil_5_20x20_460</t>
   </si>
   <si>
-    <t>Dummy</t>
-  </si>
-  <si>
-    <t>Boden</t>
-  </si>
-  <si>
     <t>(NichtAnzeigbar)</t>
   </si>
   <si>
+    <t>Normal</t>
+  </si>
+  <si>
     <t>Gekauft</t>
   </si>
   <si>
-    <t>Normal</t>
-  </si>
-  <si>
     <t>Jede</t>
   </si>
   <si>
+    <t>PART-item_0043784_Klemmwinkel 5_1-DESC</t>
+  </si>
+  <si>
+    <t>Flachrundschraube mit Vierkantansatz</t>
+  </si>
+  <si>
     <t>Unterlegscheibe</t>
   </si>
   <si>
     <t>Hutmutter</t>
-  </si>
-  <si>
-    <t>Flachrundschraube mit Vierkantansatz</t>
   </si>
   <si>
     <t>STEP AP214</t>
@@ -665,12 +674,51 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1724025</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>1724025</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="Picture 13"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="true"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId13"/>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="685800" y="904875"/>
+          <a:ext cx="1219370" cy="1219370"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="13.35546875" customWidth="true"/>
@@ -710,19 +758,16 @@
         <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F2" s="1">
-        <v>64</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" ht="68.25" customHeight="true" x14ac:dyDescent="0.25">
@@ -730,19 +775,22 @@
         <v>10</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F3" s="1">
-        <v>64</v>
+        <v>32</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="4" ht="68.25" customHeight="true" x14ac:dyDescent="0.25">
@@ -750,19 +798,19 @@
         <v>11</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F4" s="1">
-        <v>64</v>
+        <v>32</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" ht="68.25" customHeight="true" x14ac:dyDescent="0.25">
@@ -770,16 +818,19 @@
         <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F5" s="1">
-        <v>44</v>
+        <v>32</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="6" ht="68.25" customHeight="true" x14ac:dyDescent="0.25">
@@ -787,22 +838,19 @@
         <v>13</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F6" s="1">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" ht="68.25" customHeight="true" x14ac:dyDescent="0.25">
@@ -810,22 +858,22 @@
         <v>14</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F7" s="1">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" ht="68.25" customHeight="true" x14ac:dyDescent="0.25">
@@ -833,22 +881,22 @@
         <v>15</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F8" s="1">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" ht="68.25" customHeight="true" x14ac:dyDescent="0.25">
@@ -856,22 +904,22 @@
         <v>16</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F9" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" ht="68.25" customHeight="true" x14ac:dyDescent="0.25">
@@ -879,19 +927,22 @@
         <v>17</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F10" s="1">
         <v>2</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="11" ht="68.25" customHeight="true" x14ac:dyDescent="0.25">
@@ -899,22 +950,19 @@
         <v>18</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F11" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" ht="68.25" customHeight="true" x14ac:dyDescent="0.25">
@@ -922,13 +970,13 @@
         <v>19</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F12" s="1">
         <v>1</v>
@@ -939,16 +987,39 @@
         <v>20</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F13" s="1">
         <v>1</v>
+      </c>
+    </row>
+    <row r="14" ht="68.25" customHeight="true" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F14" s="1">
+        <v>1</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>